<commit_message>
chore: add new bond issue files and related documents for October 2026
</commit_message>
<xml_diff>
--- a/zrodla/nbp/bazowa.xlsx
+++ b/zrodla/nbp/bazowa.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\dane\Wydzialy\BC\Inflacja_bazowa\publikacja_internet\202608\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\dane\Wydzialy\BC\Inflacja_bazowa\publikacja_internet\202609\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193ECFB7-0A78-4109-9E32-B054B2F8572B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{948ABF3A-8822-4F86-BB18-74DFF0123B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -996,7 +996,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L315"/>
+  <dimension ref="A1:L316"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.453125" style="1" customWidth="1"/>
@@ -11822,17 +11822,39 @@
       </c>
     </row>
     <row r="311" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A311" s="4"/>
-      <c r="B311" s="13"/>
-      <c r="C311" s="5"/>
-      <c r="D311" s="5"/>
-      <c r="E311" s="5"/>
-      <c r="F311" s="5"/>
-      <c r="G311" s="13"/>
-      <c r="H311" s="5"/>
-      <c r="I311" s="5"/>
-      <c r="J311" s="5"/>
-      <c r="K311" s="6"/>
+      <c r="A311" s="27">
+        <v>46235</v>
+      </c>
+      <c r="B311" s="9">
+        <v>103.4</v>
+      </c>
+      <c r="C311" s="9">
+        <v>103.3</v>
+      </c>
+      <c r="D311" s="9">
+        <v>103.6</v>
+      </c>
+      <c r="E311" s="9">
+        <v>103.3</v>
+      </c>
+      <c r="F311" s="10">
+        <v>102.8</v>
+      </c>
+      <c r="G311" s="9">
+        <v>100.3</v>
+      </c>
+      <c r="H311" s="9">
+        <v>100.4</v>
+      </c>
+      <c r="I311" s="9">
+        <v>100.3</v>
+      </c>
+      <c r="J311" s="9">
+        <v>100.3</v>
+      </c>
+      <c r="K311" s="10">
+        <v>100.1</v>
+      </c>
     </row>
     <row r="312" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A312" s="4"/>
@@ -11849,16 +11871,12 @@
     </row>
     <row r="313" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A313" s="4"/>
-      <c r="B313" s="13" t="s">
-        <v>8</v>
-      </c>
+      <c r="B313" s="13"/>
       <c r="C313" s="5"/>
       <c r="D313" s="5"/>
       <c r="E313" s="5"/>
       <c r="F313" s="5"/>
-      <c r="G313" s="13" t="s">
-        <v>8</v>
-      </c>
+      <c r="G313" s="13"/>
       <c r="H313" s="5"/>
       <c r="I313" s="5"/>
       <c r="J313" s="5"/>
@@ -11866,18 +11884,23 @@
     </row>
     <row r="314" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A314" s="4"/>
-      <c r="B314" s="24"/>
-      <c r="C314" s="25"/>
-      <c r="D314" s="25"/>
-      <c r="E314" s="25"/>
-      <c r="F314" s="25"/>
-      <c r="G314" s="3"/>
-      <c r="H314" s="25"/>
-      <c r="I314" s="25"/>
-      <c r="J314" s="25"/>
-      <c r="K314" s="26"/>
+      <c r="B314" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C314" s="5"/>
+      <c r="D314" s="5"/>
+      <c r="E314" s="5"/>
+      <c r="F314" s="5"/>
+      <c r="G314" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="H314" s="5"/>
+      <c r="I314" s="5"/>
+      <c r="J314" s="5"/>
+      <c r="K314" s="6"/>
     </row>
     <row r="315" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A315" s="4"/>
       <c r="B315" s="24"/>
       <c r="C315" s="25"/>
       <c r="D315" s="25"/>
@@ -11888,6 +11911,18 @@
       <c r="I315" s="25"/>
       <c r="J315" s="25"/>
       <c r="K315" s="26"/>
+    </row>
+    <row r="316" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B316" s="24"/>
+      <c r="C316" s="25"/>
+      <c r="D316" s="25"/>
+      <c r="E316" s="25"/>
+      <c r="F316" s="25"/>
+      <c r="G316" s="3"/>
+      <c r="H316" s="25"/>
+      <c r="I316" s="25"/>
+      <c r="J316" s="25"/>
+      <c r="K316" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>